<commit_message>
more annotation for legacy 2025 results
</commit_message>
<xml_diff>
--- a/legacy/nola_2025_broken_results.xlsx
+++ b/legacy/nola_2025_broken_results.xlsx
@@ -102,6 +102,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Changed to 55 from 65 (bad math)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W39" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 57 from 52 based on correction to round 4 score</t>
         </r>
       </text>
     </comment>
@@ -1241,6 +1253,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1251,10 +1267,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -3650,7 +3662,7 @@
       <c r="W17" s="11" t="n">
         <v>63</v>
       </c>
-      <c r="X17" s="7" t="n">
+      <c r="X17" s="12" t="n">
         <f aca="false">N17/(N17+W17)</f>
         <v>0.511627906976744</v>
       </c>
@@ -4508,7 +4520,7 @@
       <c r="W28" s="11" t="n">
         <v>55</v>
       </c>
-      <c r="X28" s="7" t="n">
+      <c r="X28" s="12" t="n">
         <f aca="false">N28/(N28+W28)</f>
         <v>0.517543859649123</v>
       </c>
@@ -5363,12 +5375,12 @@
       <c r="V39" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="W39" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="X39" s="7" t="n">
+      <c r="W39" s="11" t="n">
+        <v>57</v>
+      </c>
+      <c r="X39" s="12" t="n">
         <f aca="false">N39/(N39+W39)</f>
-        <v>0.463917525773196</v>
+        <v>0.441176470588235</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,19 +5696,19 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="13" t="s">
         <v>171</v>
       </c>
       <c r="C45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="14" t="s">
         <v>172</v>
       </c>
       <c r="C46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14" t="s">
+      <c r="A47" s="15" t="s">
         <v>173</v>
       </c>
       <c r="C47" s="5"/>
@@ -8751,7 +8763,7 @@
       <c r="W16" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="X16" s="15" t="n">
+      <c r="X16" s="12" t="n">
         <f aca="false">N16/(N16+W16)</f>
         <v>0.447154471544715</v>
       </c>
@@ -9147,13 +9159,13 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>171</v>
       </c>
       <c r="C23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>313</v>
       </c>
       <c r="C24" s="5"/>

</xml_diff>